<commit_message>
Unify week-one content assignments and refresh IPAN scope
</commit_message>
<xml_diff>
--- a/punmicro/templates/writing/U03.xlsx
+++ b/punmicro/templates/writing/U03.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="内容编写" sheetId="1" r:id="R7c435ae33a6c46de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图片与视频" sheetId="2" r:id="R241b41ed78a6459b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEO与Schema" sheetId="3" r:id="R6c0a12cef47e46c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发检查" sheetId="4" r:id="Reabb5f17a56441b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="内容编写" sheetId="1" r:id="R73e357da34564b2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图片与视频" sheetId="2" r:id="Rda85baba0b024bba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEO与Schema" sheetId="3" r:id="Rdd31bb4153d940ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发检查" sheetId="4" r:id="R8798e563f65b4964"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -535,7 +535,7 @@
         <x:v>pun-ICON 自动菌落计数仪</x:v>
       </x:c>
       <x:c r="E8" s="11" t="str">
-        <x:v>用两三句界定已确认计数任务、目标读者与资料状态</x:v>
+        <x:v>用两三句界定已确认计数任务和目标读者，自然覆盖automated colony counter与automatic colony counter；保持同一产品页及现有标题。</x:v>
       </x:c>
       <x:c r="F8" s="11" t="str">
         <x:v>PhenoBooth+ combines colony counting with microbial fitness phenotyping on solid media.
@@ -8700,9 +8700,7 @@
       <x:c r="C20" s="3" t="str">
         <x:v>Explore pun-ICON colony counting considerations, including plate characteristics, operator review and reporting needs. Confirm details for your selected model.</x:v>
       </x:c>
-      <x:c r="D20" s="3" t="str">
-        <x:v>了解 pun-ICON 菌落计数的考虑事项，包括平板特征、操作人员复核和报告需求，并确认所选型号的具体信息。</x:v>
-      </x:c>
+      <x:c r="D20" s="3" t="str"/>
       <x:c r="E20" s="8" t="str"/>
       <x:c r="F20" s="3" t="str">
         <x:v>准确摘要，不固定字符数；搜索引擎可能重新生成片段。</x:v>
@@ -8826,9 +8824,7 @@
       <x:c r="C26" s="3" t="str">
         <x:v>Explore pun-ICON colony counting considerations, including plate characteristics, operator review and reporting needs. Confirm details for your selected model.</x:v>
       </x:c>
-      <x:c r="D26" s="3" t="str">
-        <x:v>了解 pun-ICON 菌落计数的考虑事项，包括平板特征、操作人员复核和报告需求，并确认所选型号的具体信息。</x:v>
-      </x:c>
+      <x:c r="D26" s="3" t="str"/>
       <x:c r="E26" s="8" t="str"/>
       <x:c r="F26" s="3" t="str">
         <x:v>可编辑，需与内容相符。</x:v>
@@ -8970,9 +8966,7 @@
       <x:c r="C33" s="3" t="str">
         <x:v>Explore pun-ICON colony counting considerations, including plate characteristics, operator review and reporting needs. Confirm details for your selected model.</x:v>
       </x:c>
-      <x:c r="D33" s="3" t="str">
-        <x:v>了解 pun-ICON 菌落计数的考虑事项，包括平板特征、操作人员复核和报告需求，并确认所选型号的具体信息。</x:v>
-      </x:c>
+      <x:c r="D33" s="3" t="str"/>
       <x:c r="E33" s="8" t="str"/>
       <x:c r="F33" s="3" t="str">
         <x:v>可沿用已审核摘要。</x:v>

</xml_diff>